<commit_message>
chore: format codebase and update env template for deployment
</commit_message>
<xml_diff>
--- a/test/e2e/danh_sach_sinh_vien_mau.xlsx
+++ b/test/e2e/danh_sach_sinh_vien_mau.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="DanhSachSinhVien" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Danh Sách Sinh Viên" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -22,94 +22,94 @@
     <t>Email</t>
   </si>
   <si>
-    <t>22110001</t>
+    <t>21110001</t>
   </si>
   <si>
     <t>Nguyễn Văn An</t>
   </si>
   <si>
-    <t>22110001@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110002</t>
-  </si>
-  <si>
-    <t>Trần Thị Bình</t>
-  </si>
-  <si>
-    <t>22110002@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110003</t>
+    <t>21110001@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110002</t>
+  </si>
+  <si>
+    <t>Trần Thị Bích</t>
+  </si>
+  <si>
+    <t>21110002@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110003</t>
   </si>
   <si>
     <t>Lê Hoàng Cường</t>
   </si>
   <si>
-    <t>22110003@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110004</t>
-  </si>
-  <si>
-    <t>Phạm Minh Đức</t>
-  </si>
-  <si>
-    <t>22110004@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110005</t>
-  </si>
-  <si>
-    <t>Đỗ Thị Mai</t>
-  </si>
-  <si>
-    <t>22110005@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110006</t>
-  </si>
-  <si>
-    <t>Võ Quốc Hưng</t>
-  </si>
-  <si>
-    <t>22110006@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110007</t>
-  </si>
-  <si>
-    <t>Hoàng Ngọc Lan</t>
-  </si>
-  <si>
-    <t>22110007@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110008</t>
-  </si>
-  <si>
-    <t>Bùi Thanh Phong</t>
-  </si>
-  <si>
-    <t>22110008@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110009</t>
-  </si>
-  <si>
-    <t>Đặng Khánh Linh</t>
-  </si>
-  <si>
-    <t>22110009@student.hcmute.edu.vn</t>
-  </si>
-  <si>
-    <t>22110010</t>
-  </si>
-  <si>
-    <t>Ngô Quang Huy</t>
-  </si>
-  <si>
-    <t>22110010@student.hcmute.edu.vn</t>
+    <t>21110003@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110004</t>
+  </si>
+  <si>
+    <t>Phạm Đức Dũng</t>
+  </si>
+  <si>
+    <t>21110004@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110005</t>
+  </si>
+  <si>
+    <t>Hoàng Mai Em</t>
+  </si>
+  <si>
+    <t>21110005@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110006</t>
+  </si>
+  <si>
+    <t>Vũ Quốc Phong</t>
+  </si>
+  <si>
+    <t>21110006@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110007</t>
+  </si>
+  <si>
+    <t>Đặng Thu Hà</t>
+  </si>
+  <si>
+    <t>21110007@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110008</t>
+  </si>
+  <si>
+    <t>Bùi Minh Khang</t>
+  </si>
+  <si>
+    <t>21110008@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110009</t>
+  </si>
+  <si>
+    <t>Đỗ Phương Linh</t>
+  </si>
+  <si>
+    <t>21110009@student.hcmute.edu.vn</t>
+  </si>
+  <si>
+    <t>21110010</t>
+  </si>
+  <si>
+    <t>Ngô Quang Minh</t>
+  </si>
+  <si>
+    <t>21110010@student.hcmute.edu.vn</t>
   </si>
 </sst>
 </file>
@@ -138,7 +138,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E3A8A"/>
+        <fgColor rgb="FF1E3A4A"/>
       </patternFill>
     </fill>
   </fills>
@@ -154,9 +154,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -504,7 +512,7 @@
     <col min="3" max="3" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="26" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -515,113 +523,113 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" ht="22" customHeight="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>32</v>
       </c>
     </row>

</xml_diff>